<commit_message>
Most likely displacement and support reactions work
Needs more tests to be sure. Also internal force calculations
need to be checked (one easy way would be rotating the support 90
degrees)
</commit_message>
<xml_diff>
--- a/theory/FEM matriisit.xlsx
+++ b/theory/FEM matriisit.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="821" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="825" uniqueCount="144">
   <si>
     <t xml:space="preserve">Laskenta perustuu Savonia AMK opintoihin, Ville Pekkalan opinnäytetyöhön ja netistä löytyneeseen (ei tällä hetkellä löydettävissä) Matti Lähteenmäki, Elementtimenetelmän perusteet opukseen</t>
   </si>
@@ -583,13 +583,25 @@
     <t xml:space="preserve">Yhdistetty jäykkyysmatriisi tukien kierto huomioituna</t>
   </si>
   <si>
+    <t xml:space="preserve">Kierretyt siirtymät</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kierretyt voimat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kierretyt tukireaktiot</t>
   </si>
   <si>
     <t xml:space="preserve">r22’</t>
   </si>
   <si>
     <t xml:space="preserve">r41’</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Globaalit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">siirtymät</t>
   </si>
 </sst>
 </file>
@@ -50240,10 +50252,15 @@
       <c r="AU88" s="0"/>
       <c r="AV88" s="0"/>
       <c r="AW88" s="0"/>
-      <c r="AX88" s="0"/>
+      <c r="AX88" s="0" t="s">
+        <v>137</v>
+      </c>
       <c r="AY88" s="0"/>
       <c r="AZ88" s="0" t="s">
-        <v>137</v>
+        <v>138</v>
+      </c>
+      <c r="BB88" s="0" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51116,7 +51133,7 @@
       </c>
       <c r="AQ106" s="13"/>
       <c r="AR106" s="13" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="AS106" s="13"/>
       <c r="AT106" s="21"/>
@@ -51294,7 +51311,7 @@
         <v>656250</v>
       </c>
       <c r="AR109" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="AT109" s="7"/>
       <c r="AV109" s="13"/>
@@ -51517,7 +51534,9 @@
       </c>
       <c r="AX115" s="0"/>
       <c r="AY115" s="0"/>
-      <c r="AZ115" s="7"/>
+      <c r="AZ115" s="7" t="s">
+        <v>142</v>
+      </c>
       <c r="BB115" s="7"/>
       <c r="BE115" s="7"/>
       <c r="BK115" s="21"/>
@@ -51575,6 +51594,9 @@
       </c>
       <c r="AX116" s="0"/>
       <c r="AY116" s="0"/>
+      <c r="AZ116" s="1" t="s">
+        <v>143</v>
+      </c>
       <c r="BK116" s="21"/>
       <c r="BL116" s="21"/>
       <c r="BM116" s="21"/>

</xml_diff>